<commit_message>
>= 4,000 indels everywhere (code repo ae2b1c2): ms.qmd, CLAUDE.md, Figure 4, Tables S9 and S10 legends
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BtpRPVo656vetvDm7bkL5X
</commit_message>
<xml_diff>
--- a/sup_tables/sup_table_s9_pol_proofreading.xlsx
+++ b/sup_tables/sup_table_s9_pol_proofreading.xlsx
@@ -2660,7 +2660,7 @@
     <t xml:space="preserve">Title</t>
   </si>
   <si>
-    <t xml:space="preserve">Table S9. All tumors with more than 4,000 somatic indels, with their polymerase proofreading status, their two largest indel signature exposures, and all coding mutations observed in POLD1, POLE and the mismatch-repair genes MSH2, MLH1, MSH6, PMS2 and MSH3.</t>
+    <t xml:space="preserve">Table S9. All tumors with at least 4,000 somatic indels, with their polymerase proofreading status, their two largest indel signature exposures, and all coding mutations observed in POLD1, POLE and the mismatch-repair genes MSH2, MLH1, MSH6, PMS2 and MSH3.</t>
   </si>
   <si>
     <t xml:space="preserve">Changes from the previous version</t>
@@ -2672,7 +2672,7 @@
     <t xml:space="preserve">Selection</t>
   </si>
   <si>
-    <t xml:space="preserve">More than 4,000 total somatic indels. No other criterion is applied.</t>
+    <t xml:space="preserve">At least 4,000 total somatic indels. No other criterion is applied.</t>
   </si>
   <si>
     <t xml:space="preserve">Proofreading domains</t>

</xml_diff>